<commit_message>
Elimino encuesta de percepción
La encuesta de percepción de seguridad tiene un problema de anonimización e identificación de los encuestados que no puedo resolver en este momento. Es mejor bajarla por ahora.
</commit_message>
<xml_diff>
--- a/registro_fuentes_variables.xlsx
+++ b/registro_fuentes_variables.xlsx
@@ -4268,7 +4268,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>En el repositorio</t>
+          <t>En el disco, no versionado (decisión P-18 pendiente)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -4302,7 +4302,7 @@
       <c r="L43" s="2" t="n"/>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>Anonimizado el 2026-09-17 desde Data anonimizada encuesta percepcion 2018-2025.xlsx (MD5 6899890e13175b4a0e9d0f2ef6c5ea5f): se suprimieron PD_NOMBREAUTORIZA, PD_FIRMAAUTORIZA, TELEFONO, EMAIL, DIRECCION_1, DIRECCION_1_1 y BARRIOENC. Se conservan el barrio y la comuna del marco muestral, el código de manzana, la zona, el estrato, el sexo, la edad exacta, las fechas y las respuestas abiertas, así que el riesgo de reidentificación no está eliminado (P-18). El código está en el README de la carpeta y el detalle en el anexo, sección 10.4.</t>
+          <t>Retirado del repositorio el 2026-09-17 mientras se decide P-18: la medición de riesgo mostró que 10.843 registros (46,7 %) son únicos por municipio, zona, sexo, edad exacta y estrato, y que el 97,5 % de los 7.569 registros con código de manzana es único. Queda en el disco, listado en .gitignore. Su MD5 está en esta fila, no en el manifiesto. Ojo: la versión publicada antes de esa fecha sigue en el historial de git del repositorio remoto. Anonimizado el 2026-09-17 desde Data anonimizada encuesta percepcion 2018-2025.xlsx (MD5 6899890e13175b4a0e9d0f2ef6c5ea5f): se suprimieron PD_NOMBREAUTORIZA, PD_FIRMAAUTORIZA, TELEFONO, EMAIL, DIRECCION_1, DIRECCION_1_1 y BARRIOENC. Se conservan el barrio y la comuna del marco muestral, el código de manzana, la zona, el estrato, el sexo, la edad exacta, las fechas y las respuestas abiertas, así que el riesgo de reidentificación no está eliminado (P-18). El código está en el README de la carpeta y el detalle en el anexo, sección 10.4.</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -36680,12 +36680,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Se suprimieron los identificadores directos (726 nombres, 726 firmas, 5.260 direcciones) y el barrio declarado por el encuestado (BARRIOENC, 7.599 valores distintos). Por decisión del equipo se conservaron el barrio y la comuna del marco muestral, el código de manzana (7.569 registros), la zona de muestreo, el código de entrevistador, el estrato, el sexo, la edad exacta, la fecha y la hora, y 102 columnas de respuesta abierta: en municipios pequeños esa combinación todavía permite reidentificar.</t>
+          <t>Se suprimieron los identificadores directos (726 nombres, 726 firmas, 5.260 direcciones) y el barrio declarado por el encuestado (BARRIOENC, 7.599 valores distintos). Por decisión del equipo se conservaron el barrio y la comuna del marco muestral, el código de manzana (7.569 registros), la zona de muestreo, el código de entrevistador, el estrato, el sexo, la edad exacta, la fecha y la hora, y 102 columnas de respuesta abierta: en municipios pequeños esa combinación todavía permite reidentificar. Medición hecha el 2026-09-17 sobre el parquet anonimizado (23.216 registros): con municipio, zona, sexo, edad exacta y estrato, 10.843 registros (46,7 %) son únicos y el 90,7 % está en grupos de menos de 5. Con la edad en rangos quinquenales, los únicos bajan a 1.106 (4,8 %). En los 7.569 registros con COD_MANZANA, el 97,5 % es único solo con manzana, sexo y edad exacta, y 72,5 % sigue único con la edad agrupada. En los 4.588 con BARRIO del marco muestral, 86,8 % es único. El estrato aporta poco: 14.761 registros traen 98 o 99 (sin dato).</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Medir el riesgo (por ejemplo, k-anonimato sobre municipio, manzana, sexo, edad y estrato), decidir si se generaliza más antes de compartir el archivo fuera del equipo y dejar el resultado en el README de la carpeta. Responsable por asignar.</t>
+          <t>Mientras se decide, el parquet anonimizado quedó fuera del repositorio (.gitignore). Falta: (1) decidir entre generalizar, mantener dos versiones o volver a publicarlo tal cual; (2) verificar quién tiene acceso al repositorio en GitHub; (3) decidir si se reescribe el historial para retirar la versión ya publicada; (4) dejar la decisión en el README de la carpeta. Responsable por asignar.</t>
         </is>
       </c>
     </row>
@@ -37061,7 +37061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37180,6 +37180,50 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>P-18: medición de k-anonimato sobre el parquet anonimizado y tres opciones de decisión.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>La encuesta anonimizada sale del repositorio mientras se decide P-18; el manifiesto baja a 176 archivos.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ajuste versiones de archivos
Elimino versiones de 3 archivos que tenían múltiples.
</commit_message>
<xml_diff>
--- a/registro_fuentes_variables.xlsx
+++ b/registro_fuentes_variables.xlsx
@@ -18,8 +18,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fuentes'!$A$1:$Z$182</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Variables'!$A$1:$M$321</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Brechas'!$A$1:$G$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pendientes'!$A$1:$F$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Leyenda'!$A$1:$C$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Pendientes'!$A$1:$H$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Leyenda'!$A$1:$C$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Control'!$A$1:$D$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1900,8 +1900,16 @@
           <t>Base nacional (≈19.000 filas municipio-año-área)</t>
         </is>
       </c>
-      <c r="K16" s="2" t="n"/>
-      <c r="L16" s="2" t="n"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>No vigente</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Serie anterior 1985-2035 para Antioquia. No es la misma serie en otro formato: de las 6.750 combinaciones de municipio, año y área comunes con PPED, 6.722 tienen un total distinto (diferencia relativa media 6,3 %, máxima 46 %). El equipo declaró PPED como única serie el 2026-09-17, así que el repositorio queda sin población de referencia para 1985-2017.</t>
+        </is>
+      </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Proyecciones DANE con hojas de rangos de edad (Rangos Edad Judicial, Quintenios, Otros) que podrían haber sido agregadas por el equipo. Existe otra serie DANE (PPED-AreaSexoEdadMun-2018-2042_VP.xlsx); falta definir cuál es la de referencia.</t>
@@ -1990,8 +1998,16 @@
           <t>Base nacional</t>
         </is>
       </c>
-      <c r="K17" s="2" t="n"/>
-      <c r="L17" s="2" t="n"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Actualización DANE del 30 de julio de 2025, periodo 2018-2042, que incorpora nuevas tendencias demográficas. Declarada la serie de población de referencia el 2026-09-17.</t>
+        </is>
+      </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
           <t>Original de 126 MiB: está en la carpeta de su entidad pero no se versiona (.gitignore). Lo que se versiona son sus tres hojas convertidas a parquet.</t>
@@ -2080,8 +2096,16 @@
           <t>Base nacional</t>
         </is>
       </c>
-      <c r="K18" s="2" t="n"/>
-      <c r="L18" s="2" t="n"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Conversión de la edición vigente de las proyecciones DANE (ver PPED-AreaSexoEdadMun-2018-2042_VP.xlsx).</t>
+        </is>
+      </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Convertido el 2026-09-17 desde PPED-AreaSexoEdadMun-2018-2042_VP.xlsx (hoja Índice), MD5 del original 88950d04f14dc1f70e929b1a2882bc99. El propio parquet guarda esa referencia en sus metadatos. La conversión no reproduce el archivo original byte a byte: revertirla devuelve una tabla equivalente, no el original.</t>
@@ -2174,8 +2198,16 @@
           <t>Base nacional</t>
         </is>
       </c>
-      <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Conversión de la edición vigente de las proyecciones DANE (ver PPED-AreaSexoEdadMun-2018-2042_VP.xlsx).</t>
+        </is>
+      </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Convertido el 2026-09-17 desde PPED-AreaSexoEdadMun-2018-2042_VP.xlsx (hoja PPED), MD5 del original 88950d04f14dc1f70e929b1a2882bc99. El propio parquet guarda esa referencia en sus metadatos. La conversión no reproduce el archivo original byte a byte: revertirla devuelve una tabla equivalente, no el original.</t>
@@ -2268,8 +2300,16 @@
           <t>Base nacional</t>
         </is>
       </c>
-      <c r="K20" s="2" t="n"/>
-      <c r="L20" s="2" t="n"/>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Vigente</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Conversión de la edición vigente de las proyecciones DANE (ver PPED-AreaSexoEdadMun-2018-2042_VP.xlsx).</t>
+        </is>
+      </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Convertido el 2026-09-17 desde PPED-AreaSexoEdadMun-2018-2042_VP.xlsx (hoja PobMunicipalxÁreaSexoEdad), MD5 del original 88950d04f14dc1f70e929b1a2882bc99. El propio parquet guarda esa referencia en sus metadatos. La conversión no reproduce el archivo original byte a byte: revertirla devuelve una tabla equivalente, no el original.</t>
@@ -12594,12 +12634,12 @@
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>Por confirmar</t>
+          <t>Vigente</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr">
         <is>
-          <t>Mismas 10 hojas que Mortalidad Infantil (EDA, desnutrición, etc).xls, con valores distintos.</t>
+          <t>Edición 2005-2025. Frente a Mortalidad Infantil (EDA, desnutrición, etc).xls cubre un año más y trae cifras revisadas: 478 celdas distintas en los años comunes, casi todas de ±1 caso con su tasa recalculada. Declarada vigente el 2026-09-17.</t>
         </is>
       </c>
       <c r="M143" s="2" t="n"/>
@@ -12690,12 +12730,12 @@
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>Por confirmar</t>
+          <t>No vigente</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr">
         <is>
-          <t>Mismas hojas que MORTALIDADINFMAT_ORIGINAL.xls; parece la versión actualizada.</t>
+          <t>Edición 2005-2024, anterior a MORTALIDADINFMAT_ORIGINAL.xls. Se conserva porque sustenta cifras ya publicadas.</t>
         </is>
       </c>
       <c r="M144" s="2" t="n"/>
@@ -13503,7 +13543,7 @@
       </c>
       <c r="L153" s="2" t="inlineStr">
         <is>
-          <t>Histórico IRCA nacional con hoja de Antioquia.</t>
+          <t>Histórico nacional 2007-2024 (19.160 filas, 33 departamentos) más una hoja con Antioquia. Contiene íntegramente el contenido de los otros tres archivos IRCA de esta carpeta. Declarada vigente el 2026-09-17.</t>
         </is>
       </c>
       <c r="M153" s="2" t="n"/>
@@ -13594,12 +13634,12 @@
       </c>
       <c r="K154" s="2" t="inlineStr">
         <is>
-          <t>Por confirmar</t>
+          <t>No vigente</t>
         </is>
       </c>
       <c r="L154" s="2" t="inlineStr">
         <is>
-          <t>Probable extracto de Antioquia del histórico IRCA (IRCA 2024.xlsx trae hoja histórico nacional).</t>
+          <t>Antioquia 2007-2024 (2.225 filas). Comparado celda a celda con la hoja histórico de IRCA 2024.xlsx: mismas claves y ningún valor distinto. Su contenido está incluido allí.</t>
         </is>
       </c>
       <c r="M154" s="2" t="n"/>
@@ -13690,12 +13730,12 @@
       </c>
       <c r="K155" s="2" t="inlineStr">
         <is>
-          <t>Vigente</t>
+          <t>No vigente</t>
         </is>
       </c>
       <c r="L155" s="2" t="inlineStr">
         <is>
-          <t>Corte anual 2023.</t>
+          <t>Solo 2023, 124 municipios de Antioquia. Contenido incluido en IRCA 2024.xlsx; la única diferencia es de forma: en 50 municipios este archivo deja vacío el IRCA rural donde el histórico escribe "ND".</t>
         </is>
       </c>
       <c r="M155" s="2" t="n"/>
@@ -13786,12 +13826,12 @@
       </c>
       <c r="K156" s="2" t="inlineStr">
         <is>
-          <t>Vigente</t>
+          <t>No vigente</t>
         </is>
       </c>
       <c r="L156" s="2" t="inlineStr">
         <is>
-          <t>Corte anual 2024.</t>
+          <t>Solo 2024, 124 municipios de Antioquia. Contenido incluido en IRCA 2024.xlsx, sin diferencias.</t>
         </is>
       </c>
       <c r="M156" s="2" t="n"/>
@@ -36070,7 +36110,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -36112,6 +36152,16 @@
           <t>accion</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>estado</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>fecha_cierre</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -36144,6 +36194,12 @@
           <t>Definir dónde se respaldan los tres originales pesados (almacenamiento institucional) y resolver P-18.</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -36176,6 +36232,12 @@
           <t>Construir la tabla y documentar la fuente oficial de la conformación.</t>
         </is>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -36208,6 +36270,12 @@
           <t>Asignar responsable y recuperar cada original.</t>
         </is>
       </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -36240,6 +36308,12 @@
           <t>Aplicar el protocolo de procedencia (anexo, sección 13) por lotes y por entidad.</t>
         </is>
       </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -36272,6 +36346,12 @@
           <t>Completar durante la investigación de procedencia.</t>
         </is>
       </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -36304,6 +36384,12 @@
           <t>Confirmar la entidad y mover el archivo a la carpeta de su entidad, actualizando registro y manifiesto.</t>
         </is>
       </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -36336,6 +36422,12 @@
           <t>Revisar la lista y confirmar la categoría.</t>
         </is>
       </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -36365,7 +36457,17 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Declarar la versión vigente.</t>
+          <t>IRCA 2024.xlsx y MORTALIDADINFMAT_ORIGINAL.xls quedaron declarados vigentes el 2026-09-17, con la comparación celda a celda como evidencia. Los demás archivos de cada par quedan como No vigente, sin borrarse.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Resuelto</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -36397,7 +36499,17 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Definir la serie de referencia.</t>
+          <t>El equipo declaró PPED (2018-2042) como única serie de población el 2026-09-17. POBLACION MUNICIPAL.xlsx queda No vigente; el repositorio no tiene población de referencia para 1985-2017.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Resuelto</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
@@ -36432,6 +36544,12 @@
           <t>Asignar.</t>
         </is>
       </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -36464,6 +36582,12 @@
           <t>Completar hoja_campo_original al trabajar cada fuente.</t>
         </is>
       </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -36496,6 +36620,12 @@
           <t>Asignar var_id y archivo, o retirarlas.</t>
         </is>
       </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -36528,6 +36658,12 @@
           <t>Definir la convención.</t>
         </is>
       </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -36560,6 +36696,12 @@
           <t>Definir criterio de acceso y publicación.</t>
         </is>
       </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -36592,6 +36734,12 @@
           <t>Obtener la contraseña o una copia sin cifrar de la fuente.</t>
         </is>
       </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -36624,6 +36772,12 @@
           <t>Confirmar si hace falta y solicitarlo a la Gobernación de Antioquia.</t>
         </is>
       </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -36656,6 +36810,12 @@
           <t>Definir el alcance.</t>
         </is>
       </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -36688,9 +36848,15 @@
           <t>Mientras se decide, el parquet anonimizado quedó fuera del repositorio (.gitignore). Falta: (1) decidir entre generalizar, mantener dos versiones o volver a publicarlo tal cual; (2) verificar quién tiene acceso al repositorio en GitHub; (3) decidir si se reescribe el historial para retirar la versión ya publicada; (4) dejar la decisión en el README de la carpeta. Responsable por asignar.</t>
         </is>
       </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Abierto</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F19"/>
+  <autoFilter ref="A1:H19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -36701,7 +36867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37049,8 +37215,25 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Pendientes</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>estado / fecha_cierre</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Abierto · Parcial · Resuelto, con la fecha en que se cerró. La evidencia del cierre queda en la columna de acción.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C20"/>
+  <autoFilter ref="A1:C21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -37061,7 +37244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -37224,6 +37407,28 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Versiones vigentes declaradas (IRCA, mortalidad infantil y población); hoja Pendientes con estado y fecha de cierre.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>